<commit_message>
fix(xlsx): UNI-926 FIX-FIXTURE - repair the malformed kitchen-sink row 6 and surface the save-failure reason
Refs: UNI-926
</commit_message>
<xml_diff>
--- a/docs/office/g0/fixtures/files/sheets/xlsx-kitchen-sink.xlsx
+++ b/docs/office/g0/fixtures/files/sheets/xlsx-kitchen-sink.xlsx
@@ -238,14 +238,14 @@
       </c>
     </row>
     <row r="6">
-      <c r="A5" t="s">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <f>SUM(B2:B4)</f>
         <v>4908000000</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <f>SUM(C2:C4)</f>
         <v>5408000000</v>
       </c>

</xml_diff>